<commit_message>
refactor(m71): gon man hinh M7.1 - bo khung thua, giu cach doc so
- Bo khung Tham khao ke hoach Q3 lap tay (S16 van la target M7.2), muc E Gia dinh & du lieu nen,
  khoi Tong hop file Final, nhan FINAL - CEO, dong khoa ke hoach o tieu de phieu.
- Tieu de phieu: brand - cua hang - ngay chay - so ngay. Muc Thuc te doi F -> E.
- Mo ta the chi giu cach doc so (ma tran, viec can lam, bang xep hang, bang hieu chinh);
  phieu hang muc chua cham: noi dung plan + con thieu + dau moi, bo bang 22 truong trong.
- tools/preeval_final.py: bo tien to "file Final ·" o ghi chu co che.
- So lieu va ban khoa ke hoach khong doi. Tai lieu M7.1 §0.7, §0.12 cap nhat.

QA: chot 16/17 nhu truoc (#8 co tu truoc) - tsc sach - localhost M7.1 khong NaN.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_input/04_preeval.xlsx
+++ b/data_input/04_preeval.xlsx
@@ -68377,7 +68377,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = AOV nền 282.333 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = AOV nền 282.333 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -68439,7 +68439,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = AOV nền 298.981 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = AOV nền 298.981 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -68501,7 +68501,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = AOV nền 298.981 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = AOV nền 298.981 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -68563,7 +68563,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = AOV nền 291.227 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = AOV nền 291.227 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -68625,7 +68625,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = max(AOV nền; ngưỡng × hệ số) 360.000 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = max(AOV nền; ngưỡng × hệ số) 360.000 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -68687,7 +68687,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = giá bộ món chương trình 89.000 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = giá bộ món chương trình 89.000 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -68749,7 +68749,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = AOV nền 291.227 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = AOV nền 291.227 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -68811,7 +68811,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = max(AOV nền; ngưỡng × hệ số) 600.000 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = max(AOV nền; ngưỡng × hệ số) 600.000 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -68873,7 +68873,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = AOV nền 291.227 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = AOV nền 291.227 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -68935,7 +68935,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = giá bộ món chương trình 89.000 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = giá bộ món chương trình 89.000 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -68991,7 +68991,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = TA nền × số khách tối thiểu 295.126 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = TA nền × số khách tối thiểu 295.126 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -69053,7 +69053,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = AOV nền 279.942 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = AOV nền 279.942 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -69115,7 +69115,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = nhập ở sổ 199.000 · u khách sẵn có = -49%</t>
+          <t>giá trị hoá đơn = nhập ở sổ 199.000 · u khách sẵn có = -49%</t>
         </is>
       </c>
     </row>
@@ -69177,7 +69177,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = nhập ở sổ 222.700 · u khách sẵn có = -33%</t>
+          <t>giá trị hoá đơn = nhập ở sổ 222.700 · u khách sẵn có = -33%</t>
         </is>
       </c>
     </row>
@@ -69239,7 +69239,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = nhập ở sổ 1.888.998 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = nhập ở sổ 1.888.998 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -69301,7 +69301,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = nhập ở sổ 168.114 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = nhập ở sổ 168.114 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -69363,7 +69363,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = nhập ở sổ 560.861 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = nhập ở sổ 560.861 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -69425,7 +69425,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = TA nền × số khách tối thiểu 846.229 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = TA nền × số khách tối thiểu 846.229 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -69487,7 +69487,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = AOV nền 650.223 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = AOV nền 650.223 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -69549,7 +69549,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = giá bộ món chương trình 150.000 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = giá bộ món chương trình 150.000 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -69611,7 +69611,7 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = AOV nền 650.223 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = AOV nền 650.223 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -69673,7 +69673,7 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = AOV nền 650.223 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = AOV nền 650.223 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -69735,7 +69735,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = max(AOV nền; ngưỡng × hệ số) 960.000 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = max(AOV nền; ngưỡng × hệ số) 960.000 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -69797,7 +69797,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = nhập ở sổ 690.000 · u khách sẵn có = +56%</t>
+          <t>giá trị hoá đơn = nhập ở sổ 690.000 · u khách sẵn có = +56%</t>
         </is>
       </c>
     </row>
@@ -69859,7 +69859,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = AOV nền 1.661.976 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = AOV nền 1.661.976 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -69921,7 +69921,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = nhập ở sổ 776.787 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = nhập ở sổ 776.787 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -69983,7 +69983,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = AOV nền 1.812.419 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = AOV nền 1.812.419 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -70045,7 +70045,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = TA nền × số khách tối thiểu 2.077.950 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = TA nền × số khách tối thiểu 2.077.950 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -70107,7 +70107,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = AOV nền 1.812.419 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = AOV nền 1.812.419 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -70169,7 +70169,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = nhập ở sổ 1.828.147 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = nhập ở sổ 1.828.147 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -70231,7 +70231,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = nhập ở sổ 900.000 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = nhập ở sổ 900.000 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -70293,7 +70293,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = nhập ở sổ 1.280.000 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = nhập ở sổ 1.280.000 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -70355,7 +70355,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = AOV nền 1.761.101 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = AOV nền 1.761.101 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -70417,7 +70417,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = max(AOV nền; ngưỡng × hệ số) 1.761.101 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = max(AOV nền; ngưỡng × hệ số) 1.761.101 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -70479,7 +70479,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = AOV nền 1.761.101 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = AOV nền 1.761.101 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -70541,7 +70541,7 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = nhập ở sổ 1.499.000 · u khách sẵn có = +7%</t>
+          <t>giá trị hoá đơn = nhập ở sổ 1.499.000 · u khách sẵn có = +7%</t>
         </is>
       </c>
     </row>
@@ -70603,7 +70603,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = nhập ở sổ 2.190.000 · u khách sẵn có = -27%</t>
+          <t>giá trị hoá đơn = nhập ở sổ 2.190.000 · u khách sẵn có = -27%</t>
         </is>
       </c>
     </row>
@@ -70665,7 +70665,7 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = nhập ở sổ 900.000 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = nhập ở sổ 900.000 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -70727,7 +70727,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = TA nền × số khách tối thiểu 2.780.841 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = TA nền × số khách tối thiểu 2.780.841 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>
@@ -70789,7 +70789,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>file Final · giá trị hoá đơn = nhập ở sổ 900.000 · u khách sẵn có = +0%</t>
+          <t>giá trị hoá đơn = nhập ở sổ 900.000 · u khách sẵn có = +0%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(m0,m1,m4): nap so lieu T10/2026 den 18/10 + ngan sach Q4 ban Final
- Doi ten 3 file POS T10 (hoa don, ban hang, doanh thu thang) de nhan dung thang; chay update.py -> T10 len thanh xo thang M0/M1
- M4: build-budget-q4 doc them ban NOIRE_MKT_Phan Bo Chi Phi.Q4_2026_Final (giu nhanh doc file cu)
- BudgetQ4View: cot 'Plan vs muc 2%' so phan khong gom Decoration Xmas (capBase)
- docs/modules/M4 cap nhat theo ban Final

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_input/04_preeval.xlsx
+++ b/data_input/04_preeval.xlsx
@@ -24453,10 +24453,10 @@
         <v>1619304</v>
       </c>
       <c r="X8" t="n">
-        <v>0.3768346470330426</v>
+        <v>0.3768346470327184</v>
       </c>
       <c r="Y8" t="n">
-        <v>12.05278723164535</v>
+        <v>12.05278723150992</v>
       </c>
       <c r="Z8" t="n">
         <v>0</v>
@@ -24640,10 +24640,10 @@
         <v>2698841</v>
       </c>
       <c r="X9" t="n">
-        <v>0.3768346470330409</v>
+        <v>0.3768346470327164</v>
       </c>
       <c r="Y9" t="n">
-        <v>12.05278723164529</v>
+        <v>12.05278723150986</v>
       </c>
       <c r="Z9" t="n">
         <v>0</v>
@@ -24827,10 +24827,10 @@
         <v>3778377</v>
       </c>
       <c r="X10" t="n">
-        <v>0.376834647033041</v>
+        <v>0.3768346470327163</v>
       </c>
       <c r="Y10" t="n">
-        <v>12.0527872316453</v>
+        <v>12.05278723150986</v>
       </c>
       <c r="Z10" t="n">
         <v>0</v>
@@ -44544,7 +44544,7 @@
         <v>1126986</v>
       </c>
       <c r="K42" t="n">
-        <v>0.02443344692735244</v>
+        <v>0.02443344692738264</v>
       </c>
     </row>
     <row r="43">
@@ -44584,7 +44584,7 @@
         <v>1880999</v>
       </c>
       <c r="K43" t="n">
-        <v>0.02008601939794941</v>
+        <v>0.02008601939793445</v>
       </c>
     </row>
     <row r="44">
@@ -44790,7 +44790,7 @@
         <v>1878310</v>
       </c>
       <c r="K48" t="n">
-        <v>0.04072241154558744</v>
+        <v>0.04072241154563784</v>
       </c>
     </row>
     <row r="49">
@@ -44830,7 +44830,7 @@
         <v>3134998</v>
       </c>
       <c r="K49" t="n">
-        <v>0.03347669899658209</v>
+        <v>0.03347669899655726</v>
       </c>
     </row>
     <row r="50">
@@ -45036,7 +45036,7 @@
         <v>2629634</v>
       </c>
       <c r="K54" t="n">
-        <v>0.05701137616382229</v>
+        <v>0.05701137616389288</v>
       </c>
     </row>
     <row r="55">
@@ -45076,7 +45076,7 @@
         <v>4388998</v>
       </c>
       <c r="K55" t="n">
-        <v>0.04686737859521492</v>
+        <v>0.04686737859518007</v>
       </c>
     </row>
     <row r="56">
@@ -68302,10 +68302,10 @@
         <v>202531</v>
       </c>
       <c r="L5" t="n">
-        <v>0.3612653529669584</v>
+        <v>0.3612653529672828</v>
       </c>
       <c r="M5" t="n">
-        <v>0.6387346470330415</v>
+        <v>0.6387346470327171</v>
       </c>
       <c r="N5" t="n">
         <v>17528</v>

</xml_diff>